<commit_message>
chore: add high-fidelity output plots and update gitignore
</commit_message>
<xml_diff>
--- a/outputs/papr_results.xlsx
+++ b/outputs/papr_results.xlsx
@@ -515,13 +515,13 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>7.48</v>
+        <v>7.44</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>9.75</v>
+        <v>9.82</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>10.51</v>
+        <v>10.71</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
@@ -539,16 +539,16 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5.36</v>
+        <v>5.33</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>7.03</v>
+        <v>6.98</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>7.86</v>
+        <v>7.42</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>2.72</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="4">
@@ -563,16 +563,16 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5.36</v>
+        <v>5.33</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7.03</v>
+        <v>6.98</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>7.86</v>
+        <v>7.42</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2.72</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="5">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>5.34</v>
+        <v>5.32</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7.17</v>
+        <v>6.99</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>7.64</v>
+        <v>7.41</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>2.59</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="6">
@@ -614,10 +614,10 @@
         <v>7.42</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>9.81</v>
+        <v>9.83</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>11.36</v>
+        <v>10.65</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>0</v>
@@ -635,16 +635,16 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>5.86</v>
+        <v>5.84</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>7.85</v>
+        <v>7.8</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>8.619999999999999</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.96</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="8">
@@ -659,16 +659,16 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>5.86</v>
+        <v>5.84</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>7.85</v>
+        <v>7.8</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>8.619999999999999</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1.96</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="9">
@@ -686,13 +686,13 @@
         <v>5.9</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>7.73</v>
+        <v>7.8</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>8.35</v>
+        <v>8.4</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>2.08</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="10">
@@ -707,13 +707,13 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>7.44</v>
+        <v>7.41</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>10</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>10.87</v>
+        <v>10.67</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>0</v>
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>5.95</v>
+        <v>5.96</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>7.94</v>
+        <v>7.98</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>8.630000000000001</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>2.06</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="12">
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>5.95</v>
+        <v>5.96</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>7.94</v>
+        <v>7.98</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>8.630000000000001</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>2.06</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="13">
@@ -779,16 +779,16 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>6.01</v>
+        <v>6.02</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>7.82</v>
+        <v>7.92</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>9.220000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2.17</v>
+        <v>1.87</v>
       </c>
     </row>
   </sheetData>
@@ -879,25 +879,25 @@
         <v>0.01</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>9.75</v>
+        <v>9.82</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>9.699999999999999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>7.17</v>
+        <v>6.99</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>9.76</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>7.03</v>
+        <v>6.98</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>9.68</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>7.03</v>
+        <v>6.98</v>
       </c>
       <c r="J2" s="4" t="n">
         <v>9.68</v>
@@ -913,25 +913,25 @@
         <v>0.001</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>10.51</v>
+        <v>10.71</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>10.62</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>7.64</v>
+        <v>7.41</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>10.65</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>7.86</v>
+        <v>7.42</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>10.56</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>7.86</v>
+        <v>7.42</v>
       </c>
       <c r="J3" s="4" t="n">
         <v>10.56</v>
@@ -947,25 +947,25 @@
         <v>0.01</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>9.81</v>
+        <v>9.83</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>9.76</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>7.73</v>
+        <v>7.8</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>9.74</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>7.85</v>
+        <v>7.8</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>9.68</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>7.85</v>
+        <v>7.8</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>9.68</v>
@@ -981,25 +981,25 @@
         <v>0.001</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>11.36</v>
+        <v>10.65</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>10.62</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>8.35</v>
+        <v>8.4</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>10.65</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>8.619999999999999</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>10.57</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>8.619999999999999</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>10.57</v>
@@ -1015,25 +1015,25 @@
         <v>0.01</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>10</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>9.699999999999999</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>7.82</v>
+        <v>7.92</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>9.73</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>7.94</v>
+        <v>7.98</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>9.65</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>7.94</v>
+        <v>7.98</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>9.65</v>
@@ -1049,13 +1049,13 @@
         <v>0.001</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>10.87</v>
+        <v>10.67</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>10.6</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>9.220000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>10.68</v>
@@ -1119,16 +1119,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>7.0369</v>
+        <v>7.9188</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5.6557</v>
+        <v>5.4213</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>5.6557</v>
+        <v>5.4213</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5.8432</v>
+        <v>6.1301</v>
       </c>
     </row>
     <row r="3">
@@ -1136,16 +1136,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>8.0488</v>
+        <v>7.4758</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5.8645</v>
+        <v>6.4209</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5.8645</v>
+        <v>6.4209</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5.6212</v>
+        <v>5.7391</v>
       </c>
     </row>
     <row r="4">
@@ -1153,16 +1153,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>5.856</v>
+        <v>7.3451</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5.4399</v>
+        <v>7.9069</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5.4399</v>
+        <v>7.9069</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6.1593</v>
+        <v>6.7322</v>
       </c>
     </row>
     <row r="5">
@@ -1170,16 +1170,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>6.5205</v>
+        <v>8.129200000000001</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>5.9073</v>
+        <v>4.9589</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>5.9073</v>
+        <v>4.9589</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>6.5472</v>
+        <v>6.0952</v>
       </c>
     </row>
     <row r="6">
@@ -1187,16 +1187,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7.9754</v>
+        <v>5.9831</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>6.4743</v>
+        <v>6.5297</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>6.4743</v>
+        <v>6.5297</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>6.0185</v>
+        <v>6.2601</v>
       </c>
     </row>
     <row r="7">
@@ -1204,16 +1204,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>7.1863</v>
+        <v>7.8902</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>6.1962</v>
+        <v>6.4421</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>6.1962</v>
+        <v>6.4421</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>6.0527</v>
+        <v>5.2667</v>
       </c>
     </row>
     <row r="8">
@@ -1221,16 +1221,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>7.6157</v>
+        <v>7.3113</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7.4481</v>
+        <v>5.0122</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>7.4481</v>
+        <v>5.0122</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>7.284</v>
+        <v>6.8154</v>
       </c>
     </row>
     <row r="9">
@@ -1238,16 +1238,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>8.877599999999999</v>
+        <v>8.0518</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>5.2427</v>
+        <v>5.11</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>5.2427</v>
+        <v>5.11</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5.7308</v>
+        <v>5.5861</v>
       </c>
     </row>
     <row r="10">
@@ -1255,16 +1255,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>7.671</v>
+        <v>8.0777</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>6.2606</v>
+        <v>5.9664</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>6.2606</v>
+        <v>5.9664</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>5.6297</v>
+        <v>6.4435</v>
       </c>
     </row>
     <row r="11">
@@ -1272,16 +1272,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>7.2782</v>
+        <v>5.897</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>4.8516</v>
+        <v>5.6049</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>4.8516</v>
+        <v>5.6049</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>4.6828</v>
+        <v>5.2396</v>
       </c>
     </row>
     <row r="12">
@@ -1289,16 +1289,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>8.321400000000001</v>
+        <v>6.8904</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>5.3108</v>
+        <v>4.7935</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>5.3108</v>
+        <v>4.7935</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>5.532</v>
+        <v>6.0714</v>
       </c>
     </row>
     <row r="13">
@@ -1306,16 +1306,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>7.7446</v>
+        <v>6.7538</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>5.5961</v>
+        <v>5.1464</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5.5961</v>
+        <v>5.1464</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>5.8069</v>
+        <v>6.2823</v>
       </c>
     </row>
     <row r="14">
@@ -1323,16 +1323,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>8.4137</v>
+        <v>7.0617</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>6.6726</v>
+        <v>5.8939</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6.6726</v>
+        <v>5.8939</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>5.7491</v>
+        <v>6.9018</v>
       </c>
     </row>
     <row r="15">
@@ -1340,16 +1340,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>9.5291</v>
+        <v>6.7635</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>5.6337</v>
+        <v>4.7923</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>5.6337</v>
+        <v>4.7923</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>6.552</v>
+        <v>5.82</v>
       </c>
     </row>
     <row r="16">
@@ -1357,16 +1357,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>8.8422</v>
+        <v>7.1542</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>7.172</v>
+        <v>5.7386</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>7.172</v>
+        <v>5.7386</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>6.4964</v>
+        <v>6.4278</v>
       </c>
     </row>
     <row r="17">
@@ -1374,16 +1374,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>6.6775</v>
+        <v>7.1313</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>7.8453</v>
+        <v>4.6088</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>7.8453</v>
+        <v>4.6088</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>6.0651</v>
+        <v>4.4144</v>
       </c>
     </row>
     <row r="18">
@@ -1391,16 +1391,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>7.7401</v>
+        <v>8.167</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>6.5044</v>
+        <v>5.6726</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>6.5044</v>
+        <v>5.6726</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>4.4084</v>
+        <v>4.8252</v>
       </c>
     </row>
     <row r="19">
@@ -1408,16 +1408,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>7.352</v>
+        <v>8.265000000000001</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>5.4982</v>
+        <v>4.3255</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>5.4982</v>
+        <v>4.3255</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>6.2009</v>
+        <v>5.5316</v>
       </c>
     </row>
     <row r="20">
@@ -1425,16 +1425,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>6.7398</v>
+        <v>6.8702</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>6.0799</v>
+        <v>6.4489</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>6.0799</v>
+        <v>6.4489</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>5.8312</v>
+        <v>4.6078</v>
       </c>
     </row>
     <row r="21">
@@ -1442,16 +1442,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>7.7691</v>
+        <v>7.9531</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>5.6079</v>
+        <v>4.529</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>5.6079</v>
+        <v>4.529</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>6.5323</v>
+        <v>5.6382</v>
       </c>
     </row>
     <row r="22">
@@ -1459,16 +1459,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>8.5579</v>
+        <v>8.549799999999999</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>6.3294</v>
+        <v>6.1739</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>6.3294</v>
+        <v>6.1739</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>6.3062</v>
+        <v>4.9209</v>
       </c>
     </row>
     <row r="23">
@@ -1476,16 +1476,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>7.9735</v>
+        <v>6.9998</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>4.5854</v>
+        <v>5.489</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>4.5854</v>
+        <v>5.489</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>5.8017</v>
+        <v>6.4869</v>
       </c>
     </row>
     <row r="24">
@@ -1493,16 +1493,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>7.7592</v>
+        <v>9.5342</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>5.3771</v>
+        <v>6.2936</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>5.3771</v>
+        <v>6.2936</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>7.2984</v>
+        <v>6.485</v>
       </c>
     </row>
     <row r="25">
@@ -1510,16 +1510,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>6.8859</v>
+        <v>7.3124</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>5.8033</v>
+        <v>5.6662</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>5.8033</v>
+        <v>5.6662</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>6.057</v>
+        <v>7.0929</v>
       </c>
     </row>
     <row r="26">
@@ -1527,16 +1527,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7.3829</v>
+        <v>6.1283</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>6.2249</v>
+        <v>5.6533</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>6.2249</v>
+        <v>5.6533</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>4.8271</v>
+        <v>6.2694</v>
       </c>
     </row>
     <row r="27">
@@ -1544,16 +1544,16 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>7.3335</v>
+        <v>6.4765</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>6.3227</v>
+        <v>5.4124</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>6.3227</v>
+        <v>5.4124</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>6.6676</v>
+        <v>6.5128</v>
       </c>
     </row>
     <row r="28">
@@ -1561,16 +1561,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>6.4962</v>
+        <v>10.4999</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>4.673</v>
+        <v>5.7274</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>4.673</v>
+        <v>5.7274</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>5.252</v>
+        <v>5.4201</v>
       </c>
     </row>
     <row r="29">
@@ -1578,16 +1578,16 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7.764</v>
+        <v>9.8485</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>5.644</v>
+        <v>5.5301</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>5.644</v>
+        <v>5.5301</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>6.3716</v>
+        <v>6.7099</v>
       </c>
     </row>
     <row r="30">
@@ -1595,16 +1595,16 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>7.2768</v>
+        <v>7.1783</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>5.4056</v>
+        <v>5.4012</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>5.4056</v>
+        <v>5.4012</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>6.091</v>
+        <v>6.9611</v>
       </c>
     </row>
     <row r="31">
@@ -1612,16 +1612,16 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>6.2885</v>
+        <v>7.4214</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>6.1808</v>
+        <v>6.3576</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>6.1808</v>
+        <v>6.3576</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>6.034</v>
+        <v>4.5118</v>
       </c>
     </row>
     <row r="32">
@@ -1629,16 +1629,16 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>6.8036</v>
+        <v>8.1913</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>7.1156</v>
+        <v>5.9486</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>7.1156</v>
+        <v>5.9486</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>7.2802</v>
+        <v>5.3763</v>
       </c>
     </row>
     <row r="33">
@@ -1646,16 +1646,16 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>7.169</v>
+        <v>7.6019</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>5.4045</v>
+        <v>5.8918</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>5.4045</v>
+        <v>5.8918</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>4.8681</v>
+        <v>5.5971</v>
       </c>
     </row>
     <row r="34">
@@ -1663,16 +1663,16 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>8.8028</v>
+        <v>6.6075</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>5.4448</v>
+        <v>7.304</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>5.4448</v>
+        <v>7.304</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>6.376</v>
+        <v>6.6743</v>
       </c>
     </row>
     <row r="35">
@@ -1680,16 +1680,16 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="n">
-        <v>7.7496</v>
+        <v>7.0865</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>5.6181</v>
+        <v>7.4672</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>5.6181</v>
+        <v>7.4672</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>5.695</v>
+        <v>5.6378</v>
       </c>
     </row>
     <row r="36">
@@ -1697,16 +1697,16 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="n">
-        <v>8.1111</v>
+        <v>6.4515</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>5.419</v>
+        <v>6.0151</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>5.419</v>
+        <v>6.0151</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>5.7011</v>
+        <v>6.8643</v>
       </c>
     </row>
     <row r="37">
@@ -1714,16 +1714,16 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="n">
-        <v>6.6716</v>
+        <v>9.272500000000001</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>4.915</v>
+        <v>6.777</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>4.915</v>
+        <v>6.777</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>5.5715</v>
+        <v>4.4994</v>
       </c>
     </row>
     <row r="38">
@@ -1731,16 +1731,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>9.9902</v>
+        <v>7.5265</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>4.6409</v>
+        <v>6.1044</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>4.6409</v>
+        <v>6.1044</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>5.9374</v>
+        <v>6.2331</v>
       </c>
     </row>
     <row r="39">
@@ -1748,16 +1748,16 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>7.3593</v>
+        <v>8.3337</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>4.9138</v>
+        <v>6.0065</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>4.9138</v>
+        <v>6.0065</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>5.1611</v>
+        <v>5.5343</v>
       </c>
     </row>
     <row r="40">
@@ -1765,16 +1765,16 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>7.3176</v>
+        <v>7.8547</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>5.5199</v>
+        <v>5.4088</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>5.5199</v>
+        <v>5.4088</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>5.2599</v>
+        <v>5.1696</v>
       </c>
     </row>
     <row r="41">
@@ -1782,16 +1782,16 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>7.2883</v>
+        <v>7.8816</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>5.365</v>
+        <v>5.1213</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>5.365</v>
+        <v>5.1213</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>5.8974</v>
+        <v>5.3328</v>
       </c>
     </row>
     <row r="42">
@@ -1799,16 +1799,16 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>7.6176</v>
+        <v>8.161099999999999</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>4.9009</v>
+        <v>4.8018</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>4.9009</v>
+        <v>4.8018</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>6.0335</v>
+        <v>6.3971</v>
       </c>
     </row>
     <row r="43">
@@ -1816,16 +1816,16 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>7.5151</v>
+        <v>10.2639</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>5.9641</v>
+        <v>4.4075</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>5.9641</v>
+        <v>4.4075</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>4.6907</v>
+        <v>5.6618</v>
       </c>
     </row>
     <row r="44">
@@ -1833,16 +1833,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="n">
-        <v>7.0107</v>
+        <v>5.8399</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>5.9151</v>
+        <v>6.1249</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>5.9151</v>
+        <v>6.1249</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>5.687</v>
+        <v>7.365</v>
       </c>
     </row>
     <row r="45">
@@ -1850,16 +1850,16 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>6.4373</v>
+        <v>7.4885</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>6.7429</v>
+        <v>6.8395</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>6.7429</v>
+        <v>6.8395</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>5.9795</v>
+        <v>6.2599</v>
       </c>
     </row>
     <row r="46">
@@ -1867,16 +1867,16 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>8.282999999999999</v>
+        <v>6.9264</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>6.1041</v>
+        <v>5.2326</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>6.1041</v>
+        <v>5.2326</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>5.2173</v>
+        <v>5.2712</v>
       </c>
     </row>
     <row r="47">
@@ -1884,16 +1884,16 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>8.304399999999999</v>
+        <v>7.7377</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>4.6189</v>
+        <v>4.9511</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>4.6189</v>
+        <v>4.9511</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>6.5256</v>
+        <v>5.4162</v>
       </c>
     </row>
     <row r="48">
@@ -1901,16 +1901,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>7.7908</v>
+        <v>8.252599999999999</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>5.7355</v>
+        <v>6.4893</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>5.7355</v>
+        <v>6.4893</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>7.8667</v>
+        <v>6.0693</v>
       </c>
     </row>
     <row r="49">
@@ -1918,16 +1918,16 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="n">
-        <v>7.6944</v>
+        <v>6.9715</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>5.4179</v>
+        <v>7.0781</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>5.4179</v>
+        <v>7.0781</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>6.8367</v>
+        <v>6.1805</v>
       </c>
     </row>
     <row r="50">
@@ -1935,16 +1935,16 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>8.058199999999999</v>
+        <v>7.014</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>5.7774</v>
+        <v>6.1083</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>5.7774</v>
+        <v>6.1083</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>7.6057</v>
+        <v>6.5277</v>
       </c>
     </row>
     <row r="51">
@@ -1952,16 +1952,16 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>8.5169</v>
+        <v>8.0731</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>7.0988</v>
+        <v>6.9924</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>7.0988</v>
+        <v>6.9924</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>6.8336</v>
+        <v>6.3319</v>
       </c>
     </row>
     <row r="52">
@@ -1969,16 +1969,16 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>7.5784</v>
+        <v>6.419</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>6.3507</v>
+        <v>4.8371</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>6.3507</v>
+        <v>4.8371</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>5.5571</v>
+        <v>6.4205</v>
       </c>
     </row>
     <row r="53">
@@ -1986,16 +1986,16 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>7.7402</v>
+        <v>6.7852</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>7.7504</v>
+        <v>5.7303</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>7.7504</v>
+        <v>5.7303</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>5.7657</v>
+        <v>5.3324</v>
       </c>
     </row>
     <row r="54">
@@ -2003,16 +2003,16 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>6.2264</v>
+        <v>6.7727</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>5.1945</v>
+        <v>5.5769</v>
       </c>
       <c r="D54" s="2" t="n">
-        <v>5.1945</v>
+        <v>5.5769</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>6.9584</v>
+        <v>5.012</v>
       </c>
     </row>
     <row r="55">
@@ -2020,16 +2020,16 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>10.3986</v>
+        <v>7.9873</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>5.0045</v>
+        <v>6.5678</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>5.0045</v>
+        <v>6.5678</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>6.7805</v>
+        <v>5.4922</v>
       </c>
     </row>
     <row r="56">
@@ -2037,16 +2037,16 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>8.07</v>
+        <v>6.7373</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>5.5531</v>
+        <v>4.657</v>
       </c>
       <c r="D56" s="2" t="n">
-        <v>5.5531</v>
+        <v>4.657</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>5.6668</v>
+        <v>5.5857</v>
       </c>
     </row>
     <row r="57">
@@ -2054,16 +2054,16 @@
         <v>56</v>
       </c>
       <c r="B57" s="2" t="n">
-        <v>9.774800000000001</v>
+        <v>7.9771</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>5.5612</v>
+        <v>5.5752</v>
       </c>
       <c r="D57" s="2" t="n">
-        <v>5.5612</v>
+        <v>5.5752</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>5.8259</v>
+        <v>6.4078</v>
       </c>
     </row>
     <row r="58">
@@ -2071,16 +2071,16 @@
         <v>57</v>
       </c>
       <c r="B58" s="2" t="n">
-        <v>7.3837</v>
+        <v>7.7417</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>6.9561</v>
+        <v>4.5791</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>6.9561</v>
+        <v>4.5791</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>5.025</v>
+        <v>6.7425</v>
       </c>
     </row>
     <row r="59">
@@ -2088,16 +2088,16 @@
         <v>58</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>8.4671</v>
+        <v>7.5997</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>6.78</v>
+        <v>5.2647</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>6.78</v>
+        <v>5.2647</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>5.6372</v>
+        <v>7.2563</v>
       </c>
     </row>
     <row r="60">
@@ -2105,16 +2105,16 @@
         <v>59</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>7.417</v>
+        <v>6.5992</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>7.2598</v>
+        <v>6.2597</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>7.2598</v>
+        <v>6.2597</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>4.6998</v>
+        <v>5.2482</v>
       </c>
     </row>
     <row r="61">
@@ -2122,16 +2122,16 @@
         <v>60</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>7.7843</v>
+        <v>7.6607</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>5.4744</v>
+        <v>7.348</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>5.4744</v>
+        <v>7.348</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>5.9253</v>
+        <v>6.6024</v>
       </c>
     </row>
     <row r="62">
@@ -2139,16 +2139,16 @@
         <v>61</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>5.2681</v>
+        <v>7.3368</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>6.1819</v>
+        <v>5.9446</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>6.1819</v>
+        <v>5.9446</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>5.1276</v>
+        <v>6.0394</v>
       </c>
     </row>
     <row r="63">
@@ -2156,16 +2156,16 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>7.2477</v>
+        <v>5.7576</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>5.4956</v>
+        <v>4.8527</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>5.4956</v>
+        <v>4.8527</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>4.8106</v>
+        <v>5.3135</v>
       </c>
     </row>
     <row r="64">
@@ -2173,16 +2173,16 @@
         <v>63</v>
       </c>
       <c r="B64" s="2" t="n">
-        <v>5.6428</v>
+        <v>7.5684</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>4.8661</v>
+        <v>6.2494</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>4.8661</v>
+        <v>6.2494</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>5.7407</v>
+        <v>6.0233</v>
       </c>
     </row>
     <row r="65">
@@ -2190,16 +2190,16 @@
         <v>64</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>6.4453</v>
+        <v>6.6255</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>5.5668</v>
+        <v>7.409</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>5.5668</v>
+        <v>7.409</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>4.8595</v>
+        <v>5.9321</v>
       </c>
     </row>
     <row r="66">
@@ -2207,16 +2207,16 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>5.579</v>
+        <v>7.7147</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>6.2645</v>
+        <v>6.5947</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>6.2645</v>
+        <v>6.5947</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>5.828</v>
+        <v>6.0199</v>
       </c>
     </row>
     <row r="67">
@@ -2224,16 +2224,16 @@
         <v>66</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>8.724299999999999</v>
+        <v>7.2247</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>5.9195</v>
+        <v>5.323</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>5.9195</v>
+        <v>5.323</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>7.3275</v>
+        <v>5.1052</v>
       </c>
     </row>
     <row r="68">
@@ -2241,16 +2241,16 @@
         <v>67</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>7.4095</v>
+        <v>8.8612</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>5.9803</v>
+        <v>4.4318</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>5.9803</v>
+        <v>4.4318</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>6.7567</v>
+        <v>5.3741</v>
       </c>
     </row>
     <row r="69">
@@ -2258,16 +2258,16 @@
         <v>68</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>7.2438</v>
+        <v>6.7375</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>5.8712</v>
+        <v>5.1244</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>5.8712</v>
+        <v>5.1244</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>6.0677</v>
+        <v>5.1084</v>
       </c>
     </row>
     <row r="70">
@@ -2275,16 +2275,16 @@
         <v>69</v>
       </c>
       <c r="B70" s="2" t="n">
-        <v>8.158200000000001</v>
+        <v>7.6515</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>5.2694</v>
+        <v>5.6629</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>5.2694</v>
+        <v>5.6629</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>5.7433</v>
+        <v>5.2244</v>
       </c>
     </row>
     <row r="71">
@@ -2292,16 +2292,16 @@
         <v>70</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>7.8843</v>
+        <v>7.1875</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>4.8533</v>
+        <v>6.4958</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>4.8533</v>
+        <v>6.4958</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>5.6181</v>
+        <v>5.3231</v>
       </c>
     </row>
     <row r="72">
@@ -2309,16 +2309,16 @@
         <v>71</v>
       </c>
       <c r="B72" s="2" t="n">
-        <v>7.7464</v>
+        <v>9.1754</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>5.3675</v>
+        <v>5.6628</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>5.3675</v>
+        <v>5.6628</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>6.8014</v>
+        <v>6.4479</v>
       </c>
     </row>
     <row r="73">
@@ -2326,16 +2326,16 @@
         <v>72</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>6.7811</v>
+        <v>6.8424</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>6.0817</v>
+        <v>6.4529</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>6.0817</v>
+        <v>6.4529</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>5.8232</v>
+        <v>6.1185</v>
       </c>
     </row>
     <row r="74">
@@ -2343,16 +2343,16 @@
         <v>73</v>
       </c>
       <c r="B74" s="2" t="n">
-        <v>6.8377</v>
+        <v>7.1287</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>5.12</v>
+        <v>4.8973</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>5.12</v>
+        <v>4.8973</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>6.4836</v>
+        <v>5.6744</v>
       </c>
     </row>
     <row r="75">
@@ -2360,16 +2360,16 @@
         <v>74</v>
       </c>
       <c r="B75" s="2" t="n">
-        <v>6.2709</v>
+        <v>7.4541</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>5.3728</v>
+        <v>5.8217</v>
       </c>
       <c r="D75" s="2" t="n">
-        <v>5.3728</v>
+        <v>5.8217</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>5.184</v>
+        <v>7.1482</v>
       </c>
     </row>
     <row r="76">
@@ -2377,16 +2377,16 @@
         <v>75</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>6.5003</v>
+        <v>7.5031</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>4.613</v>
+        <v>7.7914</v>
       </c>
       <c r="D76" s="2" t="n">
-        <v>4.613</v>
+        <v>7.7914</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>4.7207</v>
+        <v>5.7063</v>
       </c>
     </row>
     <row r="77">
@@ -2394,16 +2394,16 @@
         <v>76</v>
       </c>
       <c r="B77" s="2" t="n">
-        <v>6.2598</v>
+        <v>6.5861</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>6.8835</v>
+        <v>4.6339</v>
       </c>
       <c r="D77" s="2" t="n">
-        <v>6.8835</v>
+        <v>4.6339</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>6.2873</v>
+        <v>7.0006</v>
       </c>
     </row>
     <row r="78">
@@ -2411,16 +2411,16 @@
         <v>77</v>
       </c>
       <c r="B78" s="2" t="n">
-        <v>7.6615</v>
+        <v>7.511</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>5.1708</v>
+        <v>4.7787</v>
       </c>
       <c r="D78" s="2" t="n">
-        <v>5.1708</v>
+        <v>4.7787</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>5.7663</v>
+        <v>7.6581</v>
       </c>
     </row>
     <row r="79">
@@ -2428,16 +2428,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="2" t="n">
-        <v>6.8765</v>
+        <v>7.0297</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>5.8163</v>
+        <v>5.817</v>
       </c>
       <c r="D79" s="2" t="n">
-        <v>5.8163</v>
+        <v>5.817</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>5.8685</v>
+        <v>5.5235</v>
       </c>
     </row>
     <row r="80">
@@ -2445,16 +2445,16 @@
         <v>79</v>
       </c>
       <c r="B80" s="2" t="n">
-        <v>8.3774</v>
+        <v>7.3942</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>4.4878</v>
+        <v>5.7675</v>
       </c>
       <c r="D80" s="2" t="n">
-        <v>4.4878</v>
+        <v>5.7675</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>5.5631</v>
+        <v>4.8982</v>
       </c>
     </row>
     <row r="81">
@@ -2462,16 +2462,16 @@
         <v>80</v>
       </c>
       <c r="B81" s="2" t="n">
-        <v>6.3151</v>
+        <v>7.9594</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>5.2207</v>
+        <v>7.0507</v>
       </c>
       <c r="D81" s="2" t="n">
-        <v>5.2207</v>
+        <v>7.0507</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>6.2129</v>
+        <v>6.8423</v>
       </c>
     </row>
     <row r="82">
@@ -2479,16 +2479,16 @@
         <v>81</v>
       </c>
       <c r="B82" s="2" t="n">
-        <v>7.8087</v>
+        <v>9.2925</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>6.1553</v>
+        <v>5.5976</v>
       </c>
       <c r="D82" s="2" t="n">
-        <v>6.1553</v>
+        <v>5.5976</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>6.0887</v>
+        <v>5.2285</v>
       </c>
     </row>
     <row r="83">
@@ -2496,16 +2496,16 @@
         <v>82</v>
       </c>
       <c r="B83" s="2" t="n">
-        <v>7.907</v>
+        <v>7.0123</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>5.9396</v>
+        <v>6.23</v>
       </c>
       <c r="D83" s="2" t="n">
-        <v>5.9396</v>
+        <v>6.23</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>4.9766</v>
+        <v>6.1269</v>
       </c>
     </row>
     <row r="84">
@@ -2513,16 +2513,16 @@
         <v>83</v>
       </c>
       <c r="B84" s="2" t="n">
-        <v>6.0785</v>
+        <v>6.8414</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>6.429</v>
+        <v>7.4717</v>
       </c>
       <c r="D84" s="2" t="n">
-        <v>6.429</v>
+        <v>7.4717</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>6.8209</v>
+        <v>5.9458</v>
       </c>
     </row>
     <row r="85">
@@ -2530,16 +2530,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="2" t="n">
-        <v>7.48</v>
+        <v>6.2157</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>6.6564</v>
+        <v>7.2231</v>
       </c>
       <c r="D85" s="2" t="n">
-        <v>6.6564</v>
+        <v>7.2231</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>6.59</v>
+        <v>7.6943</v>
       </c>
     </row>
     <row r="86">
@@ -2547,16 +2547,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="2" t="n">
-        <v>6.9707</v>
+        <v>6.9236</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>5.9893</v>
+        <v>5.6158</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>5.9893</v>
+        <v>5.6158</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>5.3078</v>
+        <v>5.419</v>
       </c>
     </row>
     <row r="87">
@@ -2564,16 +2564,16 @@
         <v>86</v>
       </c>
       <c r="B87" s="2" t="n">
-        <v>8.467599999999999</v>
+        <v>6.2297</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>6.6939</v>
+        <v>6.1514</v>
       </c>
       <c r="D87" s="2" t="n">
-        <v>6.6939</v>
+        <v>6.1514</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>6.5274</v>
+        <v>5.1527</v>
       </c>
     </row>
     <row r="88">
@@ -2581,16 +2581,16 @@
         <v>87</v>
       </c>
       <c r="B88" s="2" t="n">
-        <v>7.1647</v>
+        <v>7.1815</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>5.7136</v>
+        <v>5.3054</v>
       </c>
       <c r="D88" s="2" t="n">
-        <v>5.7136</v>
+        <v>5.3054</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>6.3091</v>
+        <v>7.7931</v>
       </c>
     </row>
     <row r="89">
@@ -2598,16 +2598,16 @@
         <v>88</v>
       </c>
       <c r="B89" s="2" t="n">
-        <v>7.0421</v>
+        <v>7.6246</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>5.7863</v>
+        <v>5.9255</v>
       </c>
       <c r="D89" s="2" t="n">
-        <v>5.7863</v>
+        <v>5.9255</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>5.794</v>
+        <v>7.1702</v>
       </c>
     </row>
     <row r="90">
@@ -2615,16 +2615,16 @@
         <v>89</v>
       </c>
       <c r="B90" s="2" t="n">
-        <v>7.5261</v>
+        <v>6.5886</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>5.6243</v>
+        <v>5.3287</v>
       </c>
       <c r="D90" s="2" t="n">
-        <v>5.6243</v>
+        <v>5.3287</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>5.7609</v>
+        <v>6.911</v>
       </c>
     </row>
     <row r="91">
@@ -2632,16 +2632,16 @@
         <v>90</v>
       </c>
       <c r="B91" s="2" t="n">
-        <v>6.7669</v>
+        <v>6.2693</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>4.4443</v>
+        <v>5.9531</v>
       </c>
       <c r="D91" s="2" t="n">
-        <v>4.4443</v>
+        <v>5.9531</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>6.6144</v>
+        <v>7.2186</v>
       </c>
     </row>
     <row r="92">
@@ -2649,16 +2649,16 @@
         <v>91</v>
       </c>
       <c r="B92" s="2" t="n">
-        <v>6.4421</v>
+        <v>7.7584</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>6.0747</v>
+        <v>5.8898</v>
       </c>
       <c r="D92" s="2" t="n">
-        <v>6.0747</v>
+        <v>5.8898</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>5.9081</v>
+        <v>5.7175</v>
       </c>
     </row>
     <row r="93">
@@ -2666,16 +2666,16 @@
         <v>92</v>
       </c>
       <c r="B93" s="2" t="n">
-        <v>7.5152</v>
+        <v>8.726699999999999</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>5.2979</v>
+        <v>6.3383</v>
       </c>
       <c r="D93" s="2" t="n">
-        <v>5.2979</v>
+        <v>6.3383</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>5.6479</v>
+        <v>5.9566</v>
       </c>
     </row>
     <row r="94">
@@ -2683,16 +2683,16 @@
         <v>93</v>
       </c>
       <c r="B94" s="2" t="n">
-        <v>7.6658</v>
+        <v>5.8135</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>4.9059</v>
+        <v>6.2736</v>
       </c>
       <c r="D94" s="2" t="n">
-        <v>4.9059</v>
+        <v>6.2736</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>5.7783</v>
+        <v>5.6845</v>
       </c>
     </row>
     <row r="95">
@@ -2700,16 +2700,16 @@
         <v>94</v>
       </c>
       <c r="B95" s="2" t="n">
-        <v>6.954</v>
+        <v>6.1098</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>5.544</v>
+        <v>6.3155</v>
       </c>
       <c r="D95" s="2" t="n">
-        <v>5.544</v>
+        <v>6.3155</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>6.6422</v>
+        <v>6.0741</v>
       </c>
     </row>
     <row r="96">
@@ -2717,16 +2717,16 @@
         <v>95</v>
       </c>
       <c r="B96" s="2" t="n">
-        <v>8.876099999999999</v>
+        <v>7.3492</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>5.8871</v>
+        <v>5.9454</v>
       </c>
       <c r="D96" s="2" t="n">
-        <v>5.8871</v>
+        <v>5.9454</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>6.3252</v>
+        <v>5.6852</v>
       </c>
     </row>
     <row r="97">
@@ -2734,16 +2734,16 @@
         <v>96</v>
       </c>
       <c r="B97" s="2" t="n">
-        <v>6.9795</v>
+        <v>7.8936</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>5.3764</v>
+        <v>5.561</v>
       </c>
       <c r="D97" s="2" t="n">
-        <v>5.3764</v>
+        <v>5.561</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>5.405</v>
+        <v>7.2558</v>
       </c>
     </row>
     <row r="98">
@@ -2751,16 +2751,16 @@
         <v>97</v>
       </c>
       <c r="B98" s="2" t="n">
-        <v>7.2197</v>
+        <v>7.2823</v>
       </c>
       <c r="C98" s="2" t="n">
-        <v>4.2813</v>
+        <v>6.3002</v>
       </c>
       <c r="D98" s="2" t="n">
-        <v>4.2813</v>
+        <v>6.3002</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>5.5809</v>
+        <v>6.292</v>
       </c>
     </row>
     <row r="99">
@@ -2768,16 +2768,16 @@
         <v>98</v>
       </c>
       <c r="B99" s="2" t="n">
-        <v>7.46</v>
+        <v>8.0954</v>
       </c>
       <c r="C99" s="2" t="n">
-        <v>6.5684</v>
+        <v>6.0585</v>
       </c>
       <c r="D99" s="2" t="n">
-        <v>6.5684</v>
+        <v>6.0585</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>6.4404</v>
+        <v>6.441</v>
       </c>
     </row>
     <row r="100">
@@ -2785,16 +2785,16 @@
         <v>99</v>
       </c>
       <c r="B100" s="2" t="n">
-        <v>7.2687</v>
+        <v>9.005100000000001</v>
       </c>
       <c r="C100" s="2" t="n">
-        <v>5.9207</v>
+        <v>5.0174</v>
       </c>
       <c r="D100" s="2" t="n">
-        <v>5.9207</v>
+        <v>5.0174</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>5.2765</v>
+        <v>5.6942</v>
       </c>
     </row>
     <row r="101">
@@ -2802,16 +2802,16 @@
         <v>100</v>
       </c>
       <c r="B101" s="2" t="n">
-        <v>7.6285</v>
+        <v>5.4633</v>
       </c>
       <c r="C101" s="2" t="n">
-        <v>5.7514</v>
+        <v>4.5951</v>
       </c>
       <c r="D101" s="2" t="n">
-        <v>5.7514</v>
+        <v>4.5951</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>4.5492</v>
+        <v>5.1126</v>
       </c>
     </row>
     <row r="102">
@@ -2819,16 +2819,16 @@
         <v>101</v>
       </c>
       <c r="B102" s="2" t="n">
-        <v>6.4262</v>
+        <v>7.9161</v>
       </c>
       <c r="C102" s="2" t="n">
-        <v>6.0719</v>
+        <v>6.4063</v>
       </c>
       <c r="D102" s="2" t="n">
-        <v>6.0719</v>
+        <v>6.4063</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>5.1722</v>
+        <v>5.6464</v>
       </c>
     </row>
     <row r="103">
@@ -2836,16 +2836,16 @@
         <v>102</v>
       </c>
       <c r="B103" s="2" t="n">
-        <v>7.5999</v>
+        <v>6.2793</v>
       </c>
       <c r="C103" s="2" t="n">
-        <v>4.9068</v>
+        <v>7.1443</v>
       </c>
       <c r="D103" s="2" t="n">
-        <v>4.9068</v>
+        <v>7.1443</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>5.9497</v>
+        <v>5.9275</v>
       </c>
     </row>
     <row r="104">
@@ -2853,16 +2853,16 @@
         <v>103</v>
       </c>
       <c r="B104" s="2" t="n">
-        <v>6.8792</v>
+        <v>6.8158</v>
       </c>
       <c r="C104" s="2" t="n">
-        <v>5.6275</v>
+        <v>5.5331</v>
       </c>
       <c r="D104" s="2" t="n">
-        <v>5.6275</v>
+        <v>5.5331</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>6.0655</v>
+        <v>5.4126</v>
       </c>
     </row>
     <row r="105">
@@ -2870,16 +2870,16 @@
         <v>104</v>
       </c>
       <c r="B105" s="2" t="n">
-        <v>6.5476</v>
+        <v>7.7473</v>
       </c>
       <c r="C105" s="2" t="n">
-        <v>4.701</v>
+        <v>5.6275</v>
       </c>
       <c r="D105" s="2" t="n">
-        <v>4.701</v>
+        <v>5.6275</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>4.7996</v>
+        <v>5.3125</v>
       </c>
     </row>
     <row r="106">
@@ -2887,16 +2887,16 @@
         <v>105</v>
       </c>
       <c r="B106" s="2" t="n">
-        <v>9.1084</v>
+        <v>8.2661</v>
       </c>
       <c r="C106" s="2" t="n">
-        <v>6.4605</v>
+        <v>5.3947</v>
       </c>
       <c r="D106" s="2" t="n">
-        <v>6.4605</v>
+        <v>5.3947</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>5.9584</v>
+        <v>5.6608</v>
       </c>
     </row>
     <row r="107">
@@ -2904,16 +2904,16 @@
         <v>106</v>
       </c>
       <c r="B107" s="2" t="n">
-        <v>7.3764</v>
+        <v>7.2582</v>
       </c>
       <c r="C107" s="2" t="n">
-        <v>6.1415</v>
+        <v>6.5025</v>
       </c>
       <c r="D107" s="2" t="n">
-        <v>6.1415</v>
+        <v>6.5025</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>6.42</v>
+        <v>6.8489</v>
       </c>
     </row>
     <row r="108">
@@ -2921,16 +2921,16 @@
         <v>107</v>
       </c>
       <c r="B108" s="2" t="n">
-        <v>7.3787</v>
+        <v>6.863</v>
       </c>
       <c r="C108" s="2" t="n">
-        <v>5.6011</v>
+        <v>5.5003</v>
       </c>
       <c r="D108" s="2" t="n">
-        <v>5.6011</v>
+        <v>5.5003</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>4.6166</v>
+        <v>6.6997</v>
       </c>
     </row>
     <row r="109">
@@ -2938,16 +2938,16 @@
         <v>108</v>
       </c>
       <c r="B109" s="2" t="n">
-        <v>5.1722</v>
+        <v>7.2204</v>
       </c>
       <c r="C109" s="2" t="n">
-        <v>7.8896</v>
+        <v>5.3034</v>
       </c>
       <c r="D109" s="2" t="n">
-        <v>7.8896</v>
+        <v>5.3034</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>6.4081</v>
+        <v>6.6772</v>
       </c>
     </row>
     <row r="110">
@@ -2955,16 +2955,16 @@
         <v>109</v>
       </c>
       <c r="B110" s="2" t="n">
-        <v>6.7738</v>
+        <v>8.055099999999999</v>
       </c>
       <c r="C110" s="2" t="n">
-        <v>5.1284</v>
+        <v>4.9292</v>
       </c>
       <c r="D110" s="2" t="n">
-        <v>5.1284</v>
+        <v>4.9292</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>6.3018</v>
+        <v>5.1118</v>
       </c>
     </row>
     <row r="111">
@@ -2972,16 +2972,16 @@
         <v>110</v>
       </c>
       <c r="B111" s="2" t="n">
-        <v>8.375400000000001</v>
+        <v>6.1747</v>
       </c>
       <c r="C111" s="2" t="n">
-        <v>6.5778</v>
+        <v>6.0104</v>
       </c>
       <c r="D111" s="2" t="n">
-        <v>6.5778</v>
+        <v>6.0104</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>7.1676</v>
+        <v>5.457</v>
       </c>
     </row>
     <row r="112">
@@ -2989,16 +2989,16 @@
         <v>111</v>
       </c>
       <c r="B112" s="2" t="n">
-        <v>6.7601</v>
+        <v>8.4785</v>
       </c>
       <c r="C112" s="2" t="n">
-        <v>5.5156</v>
+        <v>5.4744</v>
       </c>
       <c r="D112" s="2" t="n">
-        <v>5.5156</v>
+        <v>5.4744</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>5.994</v>
+        <v>5.2767</v>
       </c>
     </row>
     <row r="113">
@@ -3006,16 +3006,16 @@
         <v>112</v>
       </c>
       <c r="B113" s="2" t="n">
-        <v>7.6649</v>
+        <v>6.7571</v>
       </c>
       <c r="C113" s="2" t="n">
-        <v>5.5118</v>
+        <v>5.641</v>
       </c>
       <c r="D113" s="2" t="n">
-        <v>5.5118</v>
+        <v>5.641</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>6.9608</v>
+        <v>4.7097</v>
       </c>
     </row>
     <row r="114">
@@ -3023,16 +3023,16 @@
         <v>113</v>
       </c>
       <c r="B114" s="2" t="n">
-        <v>7.5237</v>
+        <v>7.9794</v>
       </c>
       <c r="C114" s="2" t="n">
-        <v>5.9707</v>
+        <v>4.9214</v>
       </c>
       <c r="D114" s="2" t="n">
-        <v>5.9707</v>
+        <v>4.9214</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>7.4774</v>
+        <v>5.4578</v>
       </c>
     </row>
     <row r="115">
@@ -3040,16 +3040,16 @@
         <v>114</v>
       </c>
       <c r="B115" s="2" t="n">
-        <v>6.7931</v>
+        <v>8.3344</v>
       </c>
       <c r="C115" s="2" t="n">
-        <v>6.2485</v>
+        <v>4.8011</v>
       </c>
       <c r="D115" s="2" t="n">
-        <v>6.2485</v>
+        <v>4.8011</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>6.2376</v>
+        <v>5.5237</v>
       </c>
     </row>
     <row r="116">
@@ -3057,16 +3057,16 @@
         <v>115</v>
       </c>
       <c r="B116" s="2" t="n">
-        <v>7.0603</v>
+        <v>6.9014</v>
       </c>
       <c r="C116" s="2" t="n">
-        <v>5.7593</v>
+        <v>4.9261</v>
       </c>
       <c r="D116" s="2" t="n">
-        <v>5.7593</v>
+        <v>4.9261</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>5.224</v>
+        <v>7.0465</v>
       </c>
     </row>
     <row r="117">
@@ -3074,16 +3074,16 @@
         <v>116</v>
       </c>
       <c r="B117" s="2" t="n">
-        <v>6.7907</v>
+        <v>6.1511</v>
       </c>
       <c r="C117" s="2" t="n">
-        <v>5.9496</v>
+        <v>5.6993</v>
       </c>
       <c r="D117" s="2" t="n">
-        <v>5.9496</v>
+        <v>5.6993</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>6.5039</v>
+        <v>7.0997</v>
       </c>
     </row>
     <row r="118">
@@ -3091,16 +3091,16 @@
         <v>117</v>
       </c>
       <c r="B118" s="2" t="n">
-        <v>6.9236</v>
+        <v>7.1159</v>
       </c>
       <c r="C118" s="2" t="n">
-        <v>7.1225</v>
+        <v>5.7263</v>
       </c>
       <c r="D118" s="2" t="n">
-        <v>7.1225</v>
+        <v>5.7263</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>5.8158</v>
+        <v>7.1814</v>
       </c>
     </row>
     <row r="119">
@@ -3108,16 +3108,16 @@
         <v>118</v>
       </c>
       <c r="B119" s="2" t="n">
-        <v>8.791</v>
+        <v>6.0291</v>
       </c>
       <c r="C119" s="2" t="n">
-        <v>7.9228</v>
+        <v>5.6926</v>
       </c>
       <c r="D119" s="2" t="n">
-        <v>7.9228</v>
+        <v>5.6926</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>4.833</v>
+        <v>5.6771</v>
       </c>
     </row>
     <row r="120">
@@ -3125,16 +3125,16 @@
         <v>119</v>
       </c>
       <c r="B120" s="2" t="n">
-        <v>7.1882</v>
+        <v>7.4131</v>
       </c>
       <c r="C120" s="2" t="n">
-        <v>6.9734</v>
+        <v>5.5726</v>
       </c>
       <c r="D120" s="2" t="n">
-        <v>6.9734</v>
+        <v>5.5726</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>6.0894</v>
+        <v>5.7689</v>
       </c>
     </row>
     <row r="121">
@@ -3142,16 +3142,16 @@
         <v>120</v>
       </c>
       <c r="B121" s="2" t="n">
-        <v>7.0953</v>
+        <v>8.536799999999999</v>
       </c>
       <c r="C121" s="2" t="n">
-        <v>5.051</v>
+        <v>5.804</v>
       </c>
       <c r="D121" s="2" t="n">
-        <v>5.051</v>
+        <v>5.804</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>4.5379</v>
+        <v>5.4157</v>
       </c>
     </row>
     <row r="122">
@@ -3159,16 +3159,16 @@
         <v>121</v>
       </c>
       <c r="B122" s="2" t="n">
-        <v>7.0866</v>
+        <v>5.8944</v>
       </c>
       <c r="C122" s="2" t="n">
-        <v>5.3842</v>
+        <v>5.8718</v>
       </c>
       <c r="D122" s="2" t="n">
-        <v>5.3842</v>
+        <v>5.8718</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>6.2237</v>
+        <v>6.1801</v>
       </c>
     </row>
     <row r="123">
@@ -3176,16 +3176,16 @@
         <v>122</v>
       </c>
       <c r="B123" s="2" t="n">
-        <v>8.545500000000001</v>
+        <v>8.3804</v>
       </c>
       <c r="C123" s="2" t="n">
-        <v>6.985</v>
+        <v>6.5102</v>
       </c>
       <c r="D123" s="2" t="n">
-        <v>6.985</v>
+        <v>6.5102</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>5.062</v>
+        <v>6.7896</v>
       </c>
     </row>
     <row r="124">
@@ -3193,16 +3193,16 @@
         <v>123</v>
       </c>
       <c r="B124" s="2" t="n">
-        <v>8.0463</v>
+        <v>6.8169</v>
       </c>
       <c r="C124" s="2" t="n">
-        <v>6.0873</v>
+        <v>5.1496</v>
       </c>
       <c r="D124" s="2" t="n">
-        <v>6.0873</v>
+        <v>5.1496</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>5.2114</v>
+        <v>6.0808</v>
       </c>
     </row>
     <row r="125">
@@ -3210,16 +3210,16 @@
         <v>124</v>
       </c>
       <c r="B125" s="2" t="n">
-        <v>7.2536</v>
+        <v>9.585100000000001</v>
       </c>
       <c r="C125" s="2" t="n">
-        <v>6.3941</v>
+        <v>6.2185</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>6.3941</v>
+        <v>6.2185</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>6.1758</v>
+        <v>4.8095</v>
       </c>
     </row>
     <row r="126">
@@ -3227,16 +3227,16 @@
         <v>125</v>
       </c>
       <c r="B126" s="2" t="n">
-        <v>6.8447</v>
+        <v>7.0621</v>
       </c>
       <c r="C126" s="2" t="n">
-        <v>5.1237</v>
+        <v>5.8335</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>5.1237</v>
+        <v>5.8335</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>6.2421</v>
+        <v>6.7922</v>
       </c>
     </row>
     <row r="127">
@@ -3244,16 +3244,16 @@
         <v>126</v>
       </c>
       <c r="B127" s="2" t="n">
-        <v>6.6095</v>
+        <v>7.5162</v>
       </c>
       <c r="C127" s="2" t="n">
-        <v>5.0595</v>
+        <v>5.6864</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>5.0595</v>
+        <v>5.6864</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>5.0399</v>
+        <v>6.3357</v>
       </c>
     </row>
     <row r="128">
@@ -3261,16 +3261,16 @@
         <v>127</v>
       </c>
       <c r="B128" s="2" t="n">
-        <v>6.6626</v>
+        <v>7.4259</v>
       </c>
       <c r="C128" s="2" t="n">
-        <v>5.4621</v>
+        <v>5.0674</v>
       </c>
       <c r="D128" s="2" t="n">
-        <v>5.4621</v>
+        <v>5.0674</v>
       </c>
       <c r="E128" s="2" t="n">
-        <v>6.7845</v>
+        <v>5.677</v>
       </c>
     </row>
     <row r="129">
@@ -3278,16 +3278,16 @@
         <v>128</v>
       </c>
       <c r="B129" s="2" t="n">
-        <v>7.5437</v>
+        <v>8.2607</v>
       </c>
       <c r="C129" s="2" t="n">
-        <v>5.547</v>
+        <v>5.003</v>
       </c>
       <c r="D129" s="2" t="n">
-        <v>5.547</v>
+        <v>5.003</v>
       </c>
       <c r="E129" s="2" t="n">
-        <v>5.9807</v>
+        <v>4.3549</v>
       </c>
     </row>
     <row r="130">
@@ -3295,16 +3295,16 @@
         <v>129</v>
       </c>
       <c r="B130" s="2" t="n">
-        <v>5.9471</v>
+        <v>8.0608</v>
       </c>
       <c r="C130" s="2" t="n">
-        <v>6.8896</v>
+        <v>5.7197</v>
       </c>
       <c r="D130" s="2" t="n">
-        <v>6.8896</v>
+        <v>5.7197</v>
       </c>
       <c r="E130" s="2" t="n">
-        <v>5.7406</v>
+        <v>6.6151</v>
       </c>
     </row>
     <row r="131">
@@ -3312,16 +3312,16 @@
         <v>130</v>
       </c>
       <c r="B131" s="2" t="n">
-        <v>6.9706</v>
+        <v>6.8175</v>
       </c>
       <c r="C131" s="2" t="n">
-        <v>4.7881</v>
+        <v>6.0807</v>
       </c>
       <c r="D131" s="2" t="n">
-        <v>4.7881</v>
+        <v>6.0807</v>
       </c>
       <c r="E131" s="2" t="n">
-        <v>5.0536</v>
+        <v>5.154</v>
       </c>
     </row>
     <row r="132">
@@ -3329,16 +3329,16 @@
         <v>131</v>
       </c>
       <c r="B132" s="2" t="n">
-        <v>7.4185</v>
+        <v>8.2036</v>
       </c>
       <c r="C132" s="2" t="n">
-        <v>7.4209</v>
+        <v>7.1614</v>
       </c>
       <c r="D132" s="2" t="n">
-        <v>7.4209</v>
+        <v>7.1614</v>
       </c>
       <c r="E132" s="2" t="n">
-        <v>6.5964</v>
+        <v>5.0564</v>
       </c>
     </row>
     <row r="133">
@@ -3346,16 +3346,16 @@
         <v>132</v>
       </c>
       <c r="B133" s="2" t="n">
-        <v>7.5925</v>
+        <v>7.3553</v>
       </c>
       <c r="C133" s="2" t="n">
-        <v>5.9556</v>
+        <v>5.9406</v>
       </c>
       <c r="D133" s="2" t="n">
-        <v>5.9556</v>
+        <v>5.9406</v>
       </c>
       <c r="E133" s="2" t="n">
-        <v>4.8499</v>
+        <v>6.1973</v>
       </c>
     </row>
     <row r="134">
@@ -3363,16 +3363,16 @@
         <v>133</v>
       </c>
       <c r="B134" s="2" t="n">
-        <v>7.8006</v>
+        <v>7.1548</v>
       </c>
       <c r="C134" s="2" t="n">
-        <v>6.3341</v>
+        <v>6.6875</v>
       </c>
       <c r="D134" s="2" t="n">
-        <v>6.3341</v>
+        <v>6.6875</v>
       </c>
       <c r="E134" s="2" t="n">
-        <v>6.0566</v>
+        <v>6.7583</v>
       </c>
     </row>
     <row r="135">
@@ -3380,16 +3380,16 @@
         <v>134</v>
       </c>
       <c r="B135" s="2" t="n">
-        <v>6.6251</v>
+        <v>6.7778</v>
       </c>
       <c r="C135" s="2" t="n">
-        <v>6.0976</v>
+        <v>5.9413</v>
       </c>
       <c r="D135" s="2" t="n">
-        <v>6.0976</v>
+        <v>5.9413</v>
       </c>
       <c r="E135" s="2" t="n">
-        <v>6.266</v>
+        <v>5.5733</v>
       </c>
     </row>
     <row r="136">
@@ -3397,16 +3397,16 @@
         <v>135</v>
       </c>
       <c r="B136" s="2" t="n">
-        <v>6.6942</v>
+        <v>7.5164</v>
       </c>
       <c r="C136" s="2" t="n">
-        <v>5.2009</v>
+        <v>5.6702</v>
       </c>
       <c r="D136" s="2" t="n">
-        <v>5.2009</v>
+        <v>5.6702</v>
       </c>
       <c r="E136" s="2" t="n">
-        <v>6.9676</v>
+        <v>6.0712</v>
       </c>
     </row>
     <row r="137">
@@ -3414,16 +3414,16 @@
         <v>136</v>
       </c>
       <c r="B137" s="2" t="n">
-        <v>6.4567</v>
+        <v>6.9104</v>
       </c>
       <c r="C137" s="2" t="n">
-        <v>6.463</v>
+        <v>5.9753</v>
       </c>
       <c r="D137" s="2" t="n">
-        <v>6.463</v>
+        <v>5.9753</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>4.9318</v>
+        <v>5.7856</v>
       </c>
     </row>
     <row r="138">
@@ -3431,16 +3431,16 @@
         <v>137</v>
       </c>
       <c r="B138" s="2" t="n">
-        <v>6.4562</v>
+        <v>7.0762</v>
       </c>
       <c r="C138" s="2" t="n">
-        <v>4.2036</v>
+        <v>5.0662</v>
       </c>
       <c r="D138" s="2" t="n">
-        <v>4.2036</v>
+        <v>5.0662</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>5.2735</v>
+        <v>5.5023</v>
       </c>
     </row>
     <row r="139">
@@ -3448,16 +3448,16 @@
         <v>138</v>
       </c>
       <c r="B139" s="2" t="n">
-        <v>7.6839</v>
+        <v>7.2507</v>
       </c>
       <c r="C139" s="2" t="n">
-        <v>6.3331</v>
+        <v>5.5794</v>
       </c>
       <c r="D139" s="2" t="n">
-        <v>6.3331</v>
+        <v>5.5794</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>6.6909</v>
+        <v>5.7173</v>
       </c>
     </row>
     <row r="140">
@@ -3465,16 +3465,16 @@
         <v>139</v>
       </c>
       <c r="B140" s="2" t="n">
-        <v>7.1636</v>
+        <v>5.9883</v>
       </c>
       <c r="C140" s="2" t="n">
-        <v>5.5235</v>
+        <v>6.0654</v>
       </c>
       <c r="D140" s="2" t="n">
-        <v>5.5235</v>
+        <v>6.0654</v>
       </c>
       <c r="E140" s="2" t="n">
-        <v>6.3344</v>
+        <v>5.7828</v>
       </c>
     </row>
     <row r="141">
@@ -3482,16 +3482,16 @@
         <v>140</v>
       </c>
       <c r="B141" s="2" t="n">
-        <v>6.6935</v>
+        <v>6.2066</v>
       </c>
       <c r="C141" s="2" t="n">
-        <v>6.1101</v>
+        <v>5.2958</v>
       </c>
       <c r="D141" s="2" t="n">
-        <v>6.1101</v>
+        <v>5.2958</v>
       </c>
       <c r="E141" s="2" t="n">
-        <v>6.5775</v>
+        <v>6.7777</v>
       </c>
     </row>
     <row r="142">
@@ -3499,16 +3499,16 @@
         <v>141</v>
       </c>
       <c r="B142" s="2" t="n">
-        <v>7.3421</v>
+        <v>7.3707</v>
       </c>
       <c r="C142" s="2" t="n">
-        <v>6.7932</v>
+        <v>5.4159</v>
       </c>
       <c r="D142" s="2" t="n">
-        <v>6.7932</v>
+        <v>5.4159</v>
       </c>
       <c r="E142" s="2" t="n">
-        <v>6.0525</v>
+        <v>5.3181</v>
       </c>
     </row>
     <row r="143">
@@ -3516,16 +3516,16 @@
         <v>142</v>
       </c>
       <c r="B143" s="2" t="n">
-        <v>6.9625</v>
+        <v>6.3726</v>
       </c>
       <c r="C143" s="2" t="n">
-        <v>5.9955</v>
+        <v>4.811</v>
       </c>
       <c r="D143" s="2" t="n">
-        <v>5.9955</v>
+        <v>4.811</v>
       </c>
       <c r="E143" s="2" t="n">
-        <v>5.9305</v>
+        <v>4.6135</v>
       </c>
     </row>
     <row r="144">
@@ -3533,16 +3533,16 @@
         <v>143</v>
       </c>
       <c r="B144" s="2" t="n">
-        <v>6.8197</v>
+        <v>8.2662</v>
       </c>
       <c r="C144" s="2" t="n">
-        <v>5.6416</v>
+        <v>5.9257</v>
       </c>
       <c r="D144" s="2" t="n">
-        <v>5.6416</v>
+        <v>5.9257</v>
       </c>
       <c r="E144" s="2" t="n">
-        <v>5.2967</v>
+        <v>6.8566</v>
       </c>
     </row>
     <row r="145">
@@ -3550,16 +3550,16 @@
         <v>144</v>
       </c>
       <c r="B145" s="2" t="n">
-        <v>7.4985</v>
+        <v>7.9262</v>
       </c>
       <c r="C145" s="2" t="n">
-        <v>5.5376</v>
+        <v>6.4356</v>
       </c>
       <c r="D145" s="2" t="n">
-        <v>5.5376</v>
+        <v>6.4356</v>
       </c>
       <c r="E145" s="2" t="n">
-        <v>5.4948</v>
+        <v>6.8239</v>
       </c>
     </row>
     <row r="146">
@@ -3567,16 +3567,16 @@
         <v>145</v>
       </c>
       <c r="B146" s="2" t="n">
-        <v>6.4476</v>
+        <v>7.4926</v>
       </c>
       <c r="C146" s="2" t="n">
-        <v>5.6838</v>
+        <v>5.8531</v>
       </c>
       <c r="D146" s="2" t="n">
-        <v>5.6838</v>
+        <v>5.8531</v>
       </c>
       <c r="E146" s="2" t="n">
-        <v>6.6698</v>
+        <v>7.1882</v>
       </c>
     </row>
     <row r="147">
@@ -3584,16 +3584,16 @@
         <v>146</v>
       </c>
       <c r="B147" s="2" t="n">
-        <v>7.3589</v>
+        <v>8.9527</v>
       </c>
       <c r="C147" s="2" t="n">
-        <v>4.998</v>
+        <v>6.3219</v>
       </c>
       <c r="D147" s="2" t="n">
-        <v>4.998</v>
+        <v>6.3219</v>
       </c>
       <c r="E147" s="2" t="n">
-        <v>5.6493</v>
+        <v>5.8477</v>
       </c>
     </row>
     <row r="148">
@@ -3601,16 +3601,16 @@
         <v>147</v>
       </c>
       <c r="B148" s="2" t="n">
-        <v>8.9429</v>
+        <v>7.2242</v>
       </c>
       <c r="C148" s="2" t="n">
-        <v>6.7216</v>
+        <v>4.6198</v>
       </c>
       <c r="D148" s="2" t="n">
-        <v>6.7216</v>
+        <v>4.6198</v>
       </c>
       <c r="E148" s="2" t="n">
-        <v>5.1975</v>
+        <v>6.5076</v>
       </c>
     </row>
     <row r="149">
@@ -3618,16 +3618,16 @@
         <v>148</v>
       </c>
       <c r="B149" s="2" t="n">
-        <v>9.196999999999999</v>
+        <v>8.9099</v>
       </c>
       <c r="C149" s="2" t="n">
-        <v>5.9069</v>
+        <v>5.5786</v>
       </c>
       <c r="D149" s="2" t="n">
-        <v>5.9069</v>
+        <v>5.5786</v>
       </c>
       <c r="E149" s="2" t="n">
-        <v>5.9597</v>
+        <v>5.7619</v>
       </c>
     </row>
     <row r="150">
@@ -3635,16 +3635,16 @@
         <v>149</v>
       </c>
       <c r="B150" s="2" t="n">
-        <v>7.289</v>
+        <v>7.7699</v>
       </c>
       <c r="C150" s="2" t="n">
-        <v>4.3547</v>
+        <v>5.1695</v>
       </c>
       <c r="D150" s="2" t="n">
-        <v>4.3547</v>
+        <v>5.1695</v>
       </c>
       <c r="E150" s="2" t="n">
-        <v>4.8003</v>
+        <v>6.0145</v>
       </c>
     </row>
     <row r="151">
@@ -3652,16 +3652,16 @@
         <v>150</v>
       </c>
       <c r="B151" s="2" t="n">
-        <v>8.144600000000001</v>
+        <v>7.4559</v>
       </c>
       <c r="C151" s="2" t="n">
-        <v>4.8478</v>
+        <v>4.852</v>
       </c>
       <c r="D151" s="2" t="n">
-        <v>4.8478</v>
+        <v>4.852</v>
       </c>
       <c r="E151" s="2" t="n">
-        <v>7.8566</v>
+        <v>4.9132</v>
       </c>
     </row>
     <row r="152">
@@ -3669,16 +3669,16 @@
         <v>151</v>
       </c>
       <c r="B152" s="2" t="n">
-        <v>7.7086</v>
+        <v>6.8321</v>
       </c>
       <c r="C152" s="2" t="n">
-        <v>6.4157</v>
+        <v>4.865</v>
       </c>
       <c r="D152" s="2" t="n">
-        <v>6.4157</v>
+        <v>4.865</v>
       </c>
       <c r="E152" s="2" t="n">
-        <v>7.2443</v>
+        <v>6.4183</v>
       </c>
     </row>
     <row r="153">
@@ -3686,16 +3686,16 @@
         <v>152</v>
       </c>
       <c r="B153" s="2" t="n">
-        <v>7.2365</v>
+        <v>8.2849</v>
       </c>
       <c r="C153" s="2" t="n">
-        <v>6.8977</v>
+        <v>7.0479</v>
       </c>
       <c r="D153" s="2" t="n">
-        <v>6.8977</v>
+        <v>7.0479</v>
       </c>
       <c r="E153" s="2" t="n">
-        <v>4.7156</v>
+        <v>6.0509</v>
       </c>
     </row>
     <row r="154">
@@ -3703,16 +3703,16 @@
         <v>153</v>
       </c>
       <c r="B154" s="2" t="n">
-        <v>6.0095</v>
+        <v>8.5314</v>
       </c>
       <c r="C154" s="2" t="n">
-        <v>5.8037</v>
+        <v>5.1804</v>
       </c>
       <c r="D154" s="2" t="n">
-        <v>5.8037</v>
+        <v>5.1804</v>
       </c>
       <c r="E154" s="2" t="n">
-        <v>7.3118</v>
+        <v>6.011</v>
       </c>
     </row>
     <row r="155">
@@ -3720,16 +3720,16 @@
         <v>154</v>
       </c>
       <c r="B155" s="2" t="n">
-        <v>5.1722</v>
+        <v>7.2981</v>
       </c>
       <c r="C155" s="2" t="n">
-        <v>6.6121</v>
+        <v>5.3626</v>
       </c>
       <c r="D155" s="2" t="n">
-        <v>6.6121</v>
+        <v>5.3626</v>
       </c>
       <c r="E155" s="2" t="n">
-        <v>7.8417</v>
+        <v>6.4555</v>
       </c>
     </row>
     <row r="156">
@@ -3737,16 +3737,16 @@
         <v>155</v>
       </c>
       <c r="B156" s="2" t="n">
-        <v>6.833</v>
+        <v>6.8975</v>
       </c>
       <c r="C156" s="2" t="n">
-        <v>4.4856</v>
+        <v>5.3296</v>
       </c>
       <c r="D156" s="2" t="n">
-        <v>4.4856</v>
+        <v>5.3296</v>
       </c>
       <c r="E156" s="2" t="n">
-        <v>5.0531</v>
+        <v>4.5583</v>
       </c>
     </row>
     <row r="157">
@@ -3754,16 +3754,16 @@
         <v>156</v>
       </c>
       <c r="B157" s="2" t="n">
-        <v>7.4131</v>
+        <v>6.1954</v>
       </c>
       <c r="C157" s="2" t="n">
-        <v>6.7908</v>
+        <v>5.6885</v>
       </c>
       <c r="D157" s="2" t="n">
-        <v>6.7908</v>
+        <v>5.6885</v>
       </c>
       <c r="E157" s="2" t="n">
-        <v>5.5024</v>
+        <v>5.8521</v>
       </c>
     </row>
     <row r="158">
@@ -3771,16 +3771,16 @@
         <v>157</v>
       </c>
       <c r="B158" s="2" t="n">
-        <v>7.0984</v>
+        <v>7.3093</v>
       </c>
       <c r="C158" s="2" t="n">
-        <v>6.3444</v>
+        <v>7.2379</v>
       </c>
       <c r="D158" s="2" t="n">
-        <v>6.3444</v>
+        <v>7.2379</v>
       </c>
       <c r="E158" s="2" t="n">
-        <v>6.7909</v>
+        <v>5.9172</v>
       </c>
     </row>
     <row r="159">
@@ -3788,16 +3788,16 @@
         <v>158</v>
       </c>
       <c r="B159" s="2" t="n">
-        <v>7.0615</v>
+        <v>8.8886</v>
       </c>
       <c r="C159" s="2" t="n">
-        <v>6.2708</v>
+        <v>5.0146</v>
       </c>
       <c r="D159" s="2" t="n">
-        <v>6.2708</v>
+        <v>5.0146</v>
       </c>
       <c r="E159" s="2" t="n">
-        <v>5.5291</v>
+        <v>5.4005</v>
       </c>
     </row>
     <row r="160">
@@ -3805,16 +3805,16 @@
         <v>159</v>
       </c>
       <c r="B160" s="2" t="n">
-        <v>8.8536</v>
+        <v>6.733</v>
       </c>
       <c r="C160" s="2" t="n">
-        <v>5.2924</v>
+        <v>5.4662</v>
       </c>
       <c r="D160" s="2" t="n">
-        <v>5.2924</v>
+        <v>5.4662</v>
       </c>
       <c r="E160" s="2" t="n">
-        <v>6.6112</v>
+        <v>5.9448</v>
       </c>
     </row>
     <row r="161">
@@ -3822,16 +3822,16 @@
         <v>160</v>
       </c>
       <c r="B161" s="2" t="n">
-        <v>7.7293</v>
+        <v>9.241099999999999</v>
       </c>
       <c r="C161" s="2" t="n">
-        <v>6.3073</v>
+        <v>5.305</v>
       </c>
       <c r="D161" s="2" t="n">
-        <v>6.3073</v>
+        <v>5.305</v>
       </c>
       <c r="E161" s="2" t="n">
-        <v>6.317</v>
+        <v>6.6958</v>
       </c>
     </row>
     <row r="162">
@@ -3839,16 +3839,16 @@
         <v>161</v>
       </c>
       <c r="B162" s="2" t="n">
-        <v>7.2962</v>
+        <v>6.5271</v>
       </c>
       <c r="C162" s="2" t="n">
-        <v>5.4105</v>
+        <v>5.532</v>
       </c>
       <c r="D162" s="2" t="n">
-        <v>5.4105</v>
+        <v>5.532</v>
       </c>
       <c r="E162" s="2" t="n">
-        <v>5.6594</v>
+        <v>6.3315</v>
       </c>
     </row>
     <row r="163">
@@ -3856,16 +3856,16 @@
         <v>162</v>
       </c>
       <c r="B163" s="2" t="n">
-        <v>8.3939</v>
+        <v>7.0818</v>
       </c>
       <c r="C163" s="2" t="n">
-        <v>6.974</v>
+        <v>6.4169</v>
       </c>
       <c r="D163" s="2" t="n">
-        <v>6.974</v>
+        <v>6.4169</v>
       </c>
       <c r="E163" s="2" t="n">
-        <v>6.248</v>
+        <v>5.3921</v>
       </c>
     </row>
     <row r="164">
@@ -3873,16 +3873,16 @@
         <v>163</v>
       </c>
       <c r="B164" s="2" t="n">
-        <v>7.3288</v>
+        <v>8.051399999999999</v>
       </c>
       <c r="C164" s="2" t="n">
-        <v>6.2722</v>
+        <v>5.4372</v>
       </c>
       <c r="D164" s="2" t="n">
-        <v>6.2722</v>
+        <v>5.4372</v>
       </c>
       <c r="E164" s="2" t="n">
-        <v>7.4612</v>
+        <v>5.8979</v>
       </c>
     </row>
     <row r="165">
@@ -3890,16 +3890,16 @@
         <v>164</v>
       </c>
       <c r="B165" s="2" t="n">
-        <v>7.8044</v>
+        <v>7.3463</v>
       </c>
       <c r="C165" s="2" t="n">
-        <v>5.2517</v>
+        <v>5.7519</v>
       </c>
       <c r="D165" s="2" t="n">
-        <v>5.2517</v>
+        <v>5.7519</v>
       </c>
       <c r="E165" s="2" t="n">
-        <v>5.0428</v>
+        <v>7.5412</v>
       </c>
     </row>
     <row r="166">
@@ -3907,16 +3907,16 @@
         <v>165</v>
       </c>
       <c r="B166" s="2" t="n">
-        <v>7.4704</v>
+        <v>6.5446</v>
       </c>
       <c r="C166" s="2" t="n">
-        <v>6.5777</v>
+        <v>6.2118</v>
       </c>
       <c r="D166" s="2" t="n">
-        <v>6.5777</v>
+        <v>6.2118</v>
       </c>
       <c r="E166" s="2" t="n">
-        <v>5.1712</v>
+        <v>6.5359</v>
       </c>
     </row>
     <row r="167">
@@ -3924,16 +3924,16 @@
         <v>166</v>
       </c>
       <c r="B167" s="2" t="n">
-        <v>8.8721</v>
+        <v>7.5534</v>
       </c>
       <c r="C167" s="2" t="n">
-        <v>5.5822</v>
+        <v>6.1322</v>
       </c>
       <c r="D167" s="2" t="n">
-        <v>5.5822</v>
+        <v>6.1322</v>
       </c>
       <c r="E167" s="2" t="n">
-        <v>5.6001</v>
+        <v>6.0874</v>
       </c>
     </row>
     <row r="168">
@@ -3941,16 +3941,16 @@
         <v>167</v>
       </c>
       <c r="B168" s="2" t="n">
-        <v>6.1077</v>
+        <v>9.018800000000001</v>
       </c>
       <c r="C168" s="2" t="n">
-        <v>8.618</v>
+        <v>5.348</v>
       </c>
       <c r="D168" s="2" t="n">
-        <v>8.618</v>
+        <v>5.348</v>
       </c>
       <c r="E168" s="2" t="n">
-        <v>5.6558</v>
+        <v>6.5234</v>
       </c>
     </row>
     <row r="169">
@@ -3958,16 +3958,16 @@
         <v>168</v>
       </c>
       <c r="B169" s="2" t="n">
-        <v>6.1262</v>
+        <v>8.097099999999999</v>
       </c>
       <c r="C169" s="2" t="n">
-        <v>5.8912</v>
+        <v>5.2443</v>
       </c>
       <c r="D169" s="2" t="n">
-        <v>5.8912</v>
+        <v>5.2443</v>
       </c>
       <c r="E169" s="2" t="n">
-        <v>6.3582</v>
+        <v>5.9517</v>
       </c>
     </row>
     <row r="170">
@@ -3975,16 +3975,16 @@
         <v>169</v>
       </c>
       <c r="B170" s="2" t="n">
-        <v>6.9402</v>
+        <v>8.0442</v>
       </c>
       <c r="C170" s="2" t="n">
-        <v>6.1497</v>
+        <v>5.2883</v>
       </c>
       <c r="D170" s="2" t="n">
-        <v>6.1497</v>
+        <v>5.2883</v>
       </c>
       <c r="E170" s="2" t="n">
-        <v>5.6886</v>
+        <v>6.627</v>
       </c>
     </row>
     <row r="171">
@@ -3992,16 +3992,16 @@
         <v>170</v>
       </c>
       <c r="B171" s="2" t="n">
-        <v>8.9503</v>
+        <v>7.6151</v>
       </c>
       <c r="C171" s="2" t="n">
-        <v>5.4133</v>
+        <v>5.2759</v>
       </c>
       <c r="D171" s="2" t="n">
-        <v>5.4133</v>
+        <v>5.2759</v>
       </c>
       <c r="E171" s="2" t="n">
-        <v>5.4983</v>
+        <v>6.1353</v>
       </c>
     </row>
     <row r="172">
@@ -4009,16 +4009,16 @@
         <v>171</v>
       </c>
       <c r="B172" s="2" t="n">
-        <v>7.3184</v>
+        <v>8.711</v>
       </c>
       <c r="C172" s="2" t="n">
-        <v>4.7509</v>
+        <v>6.6093</v>
       </c>
       <c r="D172" s="2" t="n">
-        <v>4.7509</v>
+        <v>6.6093</v>
       </c>
       <c r="E172" s="2" t="n">
-        <v>5.8932</v>
+        <v>6.3885</v>
       </c>
     </row>
     <row r="173">
@@ -4026,16 +4026,16 @@
         <v>172</v>
       </c>
       <c r="B173" s="2" t="n">
-        <v>9.519</v>
+        <v>8.769299999999999</v>
       </c>
       <c r="C173" s="2" t="n">
-        <v>5.7691</v>
+        <v>4.8641</v>
       </c>
       <c r="D173" s="2" t="n">
-        <v>5.7691</v>
+        <v>4.8641</v>
       </c>
       <c r="E173" s="2" t="n">
-        <v>6.2405</v>
+        <v>6.9885</v>
       </c>
     </row>
     <row r="174">
@@ -4043,16 +4043,16 @@
         <v>173</v>
       </c>
       <c r="B174" s="2" t="n">
-        <v>5.9901</v>
+        <v>7.9144</v>
       </c>
       <c r="C174" s="2" t="n">
-        <v>5.3197</v>
+        <v>5.5476</v>
       </c>
       <c r="D174" s="2" t="n">
-        <v>5.3197</v>
+        <v>5.5476</v>
       </c>
       <c r="E174" s="2" t="n">
-        <v>6.2968</v>
+        <v>4.9697</v>
       </c>
     </row>
     <row r="175">
@@ -4060,16 +4060,16 @@
         <v>174</v>
       </c>
       <c r="B175" s="2" t="n">
-        <v>7.9431</v>
+        <v>6.8335</v>
       </c>
       <c r="C175" s="2" t="n">
-        <v>5.5125</v>
+        <v>5.5899</v>
       </c>
       <c r="D175" s="2" t="n">
-        <v>5.5125</v>
+        <v>5.5899</v>
       </c>
       <c r="E175" s="2" t="n">
-        <v>5.3638</v>
+        <v>5.2537</v>
       </c>
     </row>
     <row r="176">
@@ -4077,16 +4077,16 @@
         <v>175</v>
       </c>
       <c r="B176" s="2" t="n">
-        <v>5.863</v>
+        <v>7.0954</v>
       </c>
       <c r="C176" s="2" t="n">
-        <v>6.0464</v>
+        <v>7.835</v>
       </c>
       <c r="D176" s="2" t="n">
-        <v>6.0464</v>
+        <v>7.835</v>
       </c>
       <c r="E176" s="2" t="n">
-        <v>5.7627</v>
+        <v>5.1914</v>
       </c>
     </row>
     <row r="177">
@@ -4094,16 +4094,16 @@
         <v>176</v>
       </c>
       <c r="B177" s="2" t="n">
-        <v>6.102</v>
+        <v>9.6722</v>
       </c>
       <c r="C177" s="2" t="n">
-        <v>5.7162</v>
+        <v>5.2414</v>
       </c>
       <c r="D177" s="2" t="n">
-        <v>5.7162</v>
+        <v>5.2414</v>
       </c>
       <c r="E177" s="2" t="n">
-        <v>5.2639</v>
+        <v>6.3495</v>
       </c>
     </row>
     <row r="178">
@@ -4111,16 +4111,16 @@
         <v>177</v>
       </c>
       <c r="B178" s="2" t="n">
-        <v>7.0539</v>
+        <v>6.726</v>
       </c>
       <c r="C178" s="2" t="n">
-        <v>6.2214</v>
+        <v>6.3224</v>
       </c>
       <c r="D178" s="2" t="n">
-        <v>6.2214</v>
+        <v>6.3224</v>
       </c>
       <c r="E178" s="2" t="n">
-        <v>5.9974</v>
+        <v>5.7761</v>
       </c>
     </row>
     <row r="179">
@@ -4128,16 +4128,16 @@
         <v>178</v>
       </c>
       <c r="B179" s="2" t="n">
-        <v>6.8576</v>
+        <v>7.1056</v>
       </c>
       <c r="C179" s="2" t="n">
-        <v>5.3583</v>
+        <v>5.5032</v>
       </c>
       <c r="D179" s="2" t="n">
-        <v>5.3583</v>
+        <v>5.5032</v>
       </c>
       <c r="E179" s="2" t="n">
-        <v>5.0827</v>
+        <v>6.3214</v>
       </c>
     </row>
     <row r="180">
@@ -4145,16 +4145,16 @@
         <v>179</v>
       </c>
       <c r="B180" s="2" t="n">
-        <v>7.942</v>
+        <v>7.6455</v>
       </c>
       <c r="C180" s="2" t="n">
-        <v>5.4131</v>
+        <v>5.1285</v>
       </c>
       <c r="D180" s="2" t="n">
-        <v>5.4131</v>
+        <v>5.1285</v>
       </c>
       <c r="E180" s="2" t="n">
-        <v>5.6428</v>
+        <v>5.1085</v>
       </c>
     </row>
     <row r="181">
@@ -4162,16 +4162,16 @@
         <v>180</v>
       </c>
       <c r="B181" s="2" t="n">
-        <v>6.7544</v>
+        <v>7.8986</v>
       </c>
       <c r="C181" s="2" t="n">
-        <v>7.1307</v>
+        <v>6.5751</v>
       </c>
       <c r="D181" s="2" t="n">
-        <v>7.1307</v>
+        <v>6.5751</v>
       </c>
       <c r="E181" s="2" t="n">
-        <v>5.4762</v>
+        <v>6.0663</v>
       </c>
     </row>
     <row r="182">
@@ -4179,16 +4179,16 @@
         <v>181</v>
       </c>
       <c r="B182" s="2" t="n">
-        <v>8.8695</v>
+        <v>7.9539</v>
       </c>
       <c r="C182" s="2" t="n">
-        <v>5.4378</v>
+        <v>5.8711</v>
       </c>
       <c r="D182" s="2" t="n">
-        <v>5.4378</v>
+        <v>5.8711</v>
       </c>
       <c r="E182" s="2" t="n">
-        <v>4.6746</v>
+        <v>5.6383</v>
       </c>
     </row>
     <row r="183">
@@ -4196,16 +4196,16 @@
         <v>182</v>
       </c>
       <c r="B183" s="2" t="n">
-        <v>7.955</v>
+        <v>7.412</v>
       </c>
       <c r="C183" s="2" t="n">
-        <v>6.3024</v>
+        <v>5.5226</v>
       </c>
       <c r="D183" s="2" t="n">
-        <v>6.3024</v>
+        <v>5.5226</v>
       </c>
       <c r="E183" s="2" t="n">
-        <v>5.7184</v>
+        <v>6.1803</v>
       </c>
     </row>
     <row r="184">
@@ -4213,16 +4213,16 @@
         <v>183</v>
       </c>
       <c r="B184" s="2" t="n">
-        <v>7.6461</v>
+        <v>6.5765</v>
       </c>
       <c r="C184" s="2" t="n">
-        <v>5.9605</v>
+        <v>6.322</v>
       </c>
       <c r="D184" s="2" t="n">
-        <v>5.9605</v>
+        <v>6.322</v>
       </c>
       <c r="E184" s="2" t="n">
-        <v>5.6212</v>
+        <v>6.9111</v>
       </c>
     </row>
     <row r="185">
@@ -4230,16 +4230,16 @@
         <v>184</v>
       </c>
       <c r="B185" s="2" t="n">
-        <v>8.8399</v>
+        <v>8.2141</v>
       </c>
       <c r="C185" s="2" t="n">
-        <v>6.174</v>
+        <v>5.7735</v>
       </c>
       <c r="D185" s="2" t="n">
-        <v>6.174</v>
+        <v>5.7735</v>
       </c>
       <c r="E185" s="2" t="n">
-        <v>6.6987</v>
+        <v>5.7527</v>
       </c>
     </row>
     <row r="186">
@@ -4247,16 +4247,16 @@
         <v>185</v>
       </c>
       <c r="B186" s="2" t="n">
-        <v>8.0547</v>
+        <v>6.78</v>
       </c>
       <c r="C186" s="2" t="n">
-        <v>4.6232</v>
+        <v>5.8303</v>
       </c>
       <c r="D186" s="2" t="n">
-        <v>4.6232</v>
+        <v>5.8303</v>
       </c>
       <c r="E186" s="2" t="n">
-        <v>5.7239</v>
+        <v>4.6671</v>
       </c>
     </row>
     <row r="187">
@@ -4264,16 +4264,16 @@
         <v>186</v>
       </c>
       <c r="B187" s="2" t="n">
-        <v>5.9808</v>
+        <v>8.021599999999999</v>
       </c>
       <c r="C187" s="2" t="n">
-        <v>5.609</v>
+        <v>5.4412</v>
       </c>
       <c r="D187" s="2" t="n">
-        <v>5.609</v>
+        <v>5.4412</v>
       </c>
       <c r="E187" s="2" t="n">
-        <v>5.2999</v>
+        <v>6.5038</v>
       </c>
     </row>
     <row r="188">
@@ -4281,16 +4281,16 @@
         <v>187</v>
       </c>
       <c r="B188" s="2" t="n">
-        <v>7.323</v>
+        <v>7.2516</v>
       </c>
       <c r="C188" s="2" t="n">
-        <v>7.7787</v>
+        <v>5.5286</v>
       </c>
       <c r="D188" s="2" t="n">
-        <v>7.7787</v>
+        <v>5.5286</v>
       </c>
       <c r="E188" s="2" t="n">
-        <v>5.6371</v>
+        <v>5.0186</v>
       </c>
     </row>
     <row r="189">
@@ -4298,16 +4298,16 @@
         <v>188</v>
       </c>
       <c r="B189" s="2" t="n">
-        <v>7.9821</v>
+        <v>7.1969</v>
       </c>
       <c r="C189" s="2" t="n">
-        <v>6.4026</v>
+        <v>6.5649</v>
       </c>
       <c r="D189" s="2" t="n">
-        <v>6.4026</v>
+        <v>6.5649</v>
       </c>
       <c r="E189" s="2" t="n">
-        <v>6.5415</v>
+        <v>5.5865</v>
       </c>
     </row>
     <row r="190">
@@ -4315,16 +4315,16 @@
         <v>189</v>
       </c>
       <c r="B190" s="2" t="n">
-        <v>6.9331</v>
+        <v>6.8741</v>
       </c>
       <c r="C190" s="2" t="n">
-        <v>7.347</v>
+        <v>5.8975</v>
       </c>
       <c r="D190" s="2" t="n">
-        <v>7.347</v>
+        <v>5.8975</v>
       </c>
       <c r="E190" s="2" t="n">
-        <v>6.3921</v>
+        <v>5.8563</v>
       </c>
     </row>
     <row r="191">
@@ -4332,16 +4332,16 @@
         <v>190</v>
       </c>
       <c r="B191" s="2" t="n">
-        <v>8.100099999999999</v>
+        <v>7.8308</v>
       </c>
       <c r="C191" s="2" t="n">
-        <v>5.5963</v>
+        <v>7.4383</v>
       </c>
       <c r="D191" s="2" t="n">
-        <v>5.5963</v>
+        <v>7.4383</v>
       </c>
       <c r="E191" s="2" t="n">
-        <v>5.5791</v>
+        <v>7.4306</v>
       </c>
     </row>
     <row r="192">
@@ -4349,16 +4349,16 @@
         <v>191</v>
       </c>
       <c r="B192" s="2" t="n">
-        <v>6.1367</v>
+        <v>7.8619</v>
       </c>
       <c r="C192" s="2" t="n">
-        <v>6.7028</v>
+        <v>6.2949</v>
       </c>
       <c r="D192" s="2" t="n">
-        <v>6.7028</v>
+        <v>6.2949</v>
       </c>
       <c r="E192" s="2" t="n">
-        <v>5.7119</v>
+        <v>5.4185</v>
       </c>
     </row>
     <row r="193">
@@ -4366,16 +4366,16 @@
         <v>192</v>
       </c>
       <c r="B193" s="2" t="n">
-        <v>8.2019</v>
+        <v>7.8757</v>
       </c>
       <c r="C193" s="2" t="n">
-        <v>5.0535</v>
+        <v>5.7791</v>
       </c>
       <c r="D193" s="2" t="n">
-        <v>5.0535</v>
+        <v>5.7791</v>
       </c>
       <c r="E193" s="2" t="n">
-        <v>4.9546</v>
+        <v>5.0606</v>
       </c>
     </row>
     <row r="194">
@@ -4383,16 +4383,16 @@
         <v>193</v>
       </c>
       <c r="B194" s="2" t="n">
-        <v>8.934200000000001</v>
+        <v>7.586</v>
       </c>
       <c r="C194" s="2" t="n">
-        <v>6.4397</v>
+        <v>5.9965</v>
       </c>
       <c r="D194" s="2" t="n">
-        <v>6.4397</v>
+        <v>5.9965</v>
       </c>
       <c r="E194" s="2" t="n">
-        <v>4.7739</v>
+        <v>5.3724</v>
       </c>
     </row>
     <row r="195">
@@ -4400,16 +4400,16 @@
         <v>194</v>
       </c>
       <c r="B195" s="2" t="n">
-        <v>7.5726</v>
+        <v>7.5384</v>
       </c>
       <c r="C195" s="2" t="n">
-        <v>5.8943</v>
+        <v>6.1717</v>
       </c>
       <c r="D195" s="2" t="n">
-        <v>5.8943</v>
+        <v>6.1717</v>
       </c>
       <c r="E195" s="2" t="n">
-        <v>5.0638</v>
+        <v>6.5842</v>
       </c>
     </row>
     <row r="196">
@@ -4417,16 +4417,16 @@
         <v>195</v>
       </c>
       <c r="B196" s="2" t="n">
-        <v>6.9302</v>
+        <v>6.0156</v>
       </c>
       <c r="C196" s="2" t="n">
-        <v>5.3825</v>
+        <v>6.925</v>
       </c>
       <c r="D196" s="2" t="n">
-        <v>5.3825</v>
+        <v>6.925</v>
       </c>
       <c r="E196" s="2" t="n">
-        <v>5.5995</v>
+        <v>5.791</v>
       </c>
     </row>
     <row r="197">
@@ -4434,16 +4434,16 @@
         <v>196</v>
       </c>
       <c r="B197" s="2" t="n">
-        <v>7.4388</v>
+        <v>8.5816</v>
       </c>
       <c r="C197" s="2" t="n">
-        <v>5.3061</v>
+        <v>6.3979</v>
       </c>
       <c r="D197" s="2" t="n">
-        <v>5.3061</v>
+        <v>6.3979</v>
       </c>
       <c r="E197" s="2" t="n">
-        <v>6.7131</v>
+        <v>5.446</v>
       </c>
     </row>
     <row r="198">
@@ -4451,16 +4451,16 @@
         <v>197</v>
       </c>
       <c r="B198" s="2" t="n">
-        <v>8.3969</v>
+        <v>6.4431</v>
       </c>
       <c r="C198" s="2" t="n">
-        <v>4.865</v>
+        <v>4.922</v>
       </c>
       <c r="D198" s="2" t="n">
-        <v>4.865</v>
+        <v>4.922</v>
       </c>
       <c r="E198" s="2" t="n">
-        <v>6.2769</v>
+        <v>5.7639</v>
       </c>
     </row>
     <row r="199">
@@ -4468,16 +4468,16 @@
         <v>198</v>
       </c>
       <c r="B199" s="2" t="n">
-        <v>7.1112</v>
+        <v>6.1556</v>
       </c>
       <c r="C199" s="2" t="n">
-        <v>6.2368</v>
+        <v>6.4866</v>
       </c>
       <c r="D199" s="2" t="n">
-        <v>6.2368</v>
+        <v>6.4866</v>
       </c>
       <c r="E199" s="2" t="n">
-        <v>5.736</v>
+        <v>5.0613</v>
       </c>
     </row>
     <row r="200">
@@ -4485,16 +4485,16 @@
         <v>199</v>
       </c>
       <c r="B200" s="2" t="n">
-        <v>7.7183</v>
+        <v>6.3802</v>
       </c>
       <c r="C200" s="2" t="n">
-        <v>5.8466</v>
+        <v>6.0423</v>
       </c>
       <c r="D200" s="2" t="n">
-        <v>5.8466</v>
+        <v>6.0423</v>
       </c>
       <c r="E200" s="2" t="n">
-        <v>5.1846</v>
+        <v>4.5044</v>
       </c>
     </row>
     <row r="201">
@@ -4502,16 +4502,16 @@
         <v>200</v>
       </c>
       <c r="B201" s="2" t="n">
-        <v>5.9609</v>
+        <v>6.534</v>
       </c>
       <c r="C201" s="2" t="n">
-        <v>6.8668</v>
+        <v>6.2702</v>
       </c>
       <c r="D201" s="2" t="n">
-        <v>6.8668</v>
+        <v>6.2702</v>
       </c>
       <c r="E201" s="2" t="n">
-        <v>6.3004</v>
+        <v>5.9298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>